<commit_message>
completed 11 test cases for UAT functionality completed 3 test cases for RnR functionality
</commit_message>
<xml_diff>
--- a/src/main/resources/UATAnnouncement_Field_Values.xlsx
+++ b/src/main/resources/UATAnnouncement_Field_Values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workpace-gov-grants-framework-automation\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45FF716A-FE61-46AC-8CA9-3E7609B883BF}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA6CDC4D-BE39-4E17-A56C-D8301E8B8E5C}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="6" activeTab="9" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="10" activeTab="12" xr2:uid="{D00E3ABE-F797-4780-AECA-E481BEE93CAC}"/>
   </bookViews>
   <sheets>
     <sheet name="DirectedAnnouncement" sheetId="1" r:id="rId1"/>
@@ -23,22 +23,26 @@
     <sheet name="FormulaAnnouncement" sheetId="8" r:id="rId8"/>
     <sheet name="Creation" sheetId="7" r:id="rId9"/>
     <sheet name="Edition" sheetId="2" r:id="rId10"/>
-    <sheet name="AppDueDate" sheetId="20" r:id="rId11"/>
-    <sheet name="Edition1" sheetId="10" r:id="rId12"/>
-    <sheet name="PreAppDueDate" sheetId="21" r:id="rId13"/>
-    <sheet name="BudgetPeriod" sheetId="3" r:id="rId14"/>
-    <sheet name="Reviewer" sheetId="4" r:id="rId15"/>
-    <sheet name="Creation Second Modal" sheetId="6" r:id="rId16"/>
-    <sheet name="Creation Second Modal for App" sheetId="25" r:id="rId17"/>
-    <sheet name="Creation Second Modal FA" sheetId="24" r:id="rId18"/>
-    <sheet name="Creation Second Modal1" sheetId="14" r:id="rId19"/>
-    <sheet name="Creation Second Modal3" sheetId="17" r:id="rId20"/>
-    <sheet name="Creation Second Modal4" sheetId="18" r:id="rId21"/>
-    <sheet name="Creation of Second Modal" sheetId="15" r:id="rId22"/>
-    <sheet name="EnterReview" sheetId="9" r:id="rId23"/>
-    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId24"/>
-    <sheet name="Edition2" sheetId="12" r:id="rId25"/>
-    <sheet name="RiskAssessmentNo" sheetId="13" r:id="rId26"/>
+    <sheet name="UATPackageCreation" sheetId="29" r:id="rId11"/>
+    <sheet name="UATTermsConditionCreation" sheetId="30" r:id="rId12"/>
+    <sheet name="UATProgramCreation" sheetId="31" r:id="rId13"/>
+    <sheet name="UATProgramEdition" sheetId="32" r:id="rId14"/>
+    <sheet name="AppDueDate" sheetId="20" r:id="rId15"/>
+    <sheet name="Edition1" sheetId="10" r:id="rId16"/>
+    <sheet name="PreAppDueDate" sheetId="21" r:id="rId17"/>
+    <sheet name="BudgetPeriod" sheetId="3" r:id="rId18"/>
+    <sheet name="Reviewer" sheetId="4" r:id="rId19"/>
+    <sheet name="Creation Second Modal" sheetId="6" r:id="rId20"/>
+    <sheet name="Creation Second Modal for App" sheetId="25" r:id="rId21"/>
+    <sheet name="Creation Second Modal FA" sheetId="24" r:id="rId22"/>
+    <sheet name="Creation Second Modal1" sheetId="14" r:id="rId23"/>
+    <sheet name="Creation Second Modal3" sheetId="17" r:id="rId24"/>
+    <sheet name="Creation Second Modal4" sheetId="18" r:id="rId25"/>
+    <sheet name="Creation of Second Modal" sheetId="15" r:id="rId26"/>
+    <sheet name="EnterReview" sheetId="9" r:id="rId27"/>
+    <sheet name="Pre-Application Modal" sheetId="11" r:id="rId28"/>
+    <sheet name="Edition2" sheetId="12" r:id="rId29"/>
+    <sheet name="RiskAssessmentNo" sheetId="13" r:id="rId30"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -50,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="681" uniqueCount="96">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -251,6 +255,93 @@
   </si>
   <si>
     <t>fieldPreApplicationDueDate__c</t>
+  </si>
+  <si>
+    <t>fieldName</t>
+  </si>
+  <si>
+    <t>fieldGNT__CustomAppConfig__c</t>
+  </si>
+  <si>
+    <t>fieldGNT__SubmissionType__c</t>
+  </si>
+  <si>
+    <t>fieldGNT__Status__c</t>
+  </si>
+  <si>
+    <t>StateasGrantor</t>
+  </si>
+  <si>
+    <t>Application</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Automation Runtime Package</t>
+  </si>
+  <si>
+    <t>fieldTitle__c</t>
+  </si>
+  <si>
+    <t>fieldTermType__c</t>
+  </si>
+  <si>
+    <t>fieldEffectiveFrom__c</t>
+  </si>
+  <si>
+    <t>fieldEffectiveTill__c</t>
+  </si>
+  <si>
+    <t>fieldStatus__c</t>
+  </si>
+  <si>
+    <t>fieldDescription__c</t>
+  </si>
+  <si>
+    <t>Automation Runtime Terms and Condition</t>
+  </si>
+  <si>
+    <t>Term</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Automation Terms</t>
+  </si>
+  <si>
+    <t>ProgramName__c</t>
+  </si>
+  <si>
+    <t>Automation Runtime Internal Program</t>
+  </si>
+  <si>
+    <t>Type__c</t>
+  </si>
+  <si>
+    <t>Project Grants</t>
+  </si>
+  <si>
+    <t>PrimaryFundingOrganization__c</t>
+  </si>
+  <si>
+    <t>Test Automation Organization</t>
+  </si>
+  <si>
+    <t>Abbreviation__c</t>
+  </si>
+  <si>
+    <t>PREG</t>
+  </si>
+  <si>
+    <t>WebsiteAddress__c</t>
+  </si>
+  <si>
+    <t>http://automate.com</t>
+  </si>
+  <si>
+    <t>Objectives__c</t>
   </si>
 </sst>
 </file>
@@ -865,6 +956,323 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20F93AC1-193C-4008-88FA-912F07544036}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="8.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.06640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68487F44-505C-4EB3-B208-49F67A1A5E36}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="7.265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.53125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="35.73046875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{867C018A-0140-4226-84B4-72270EE09F41}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="27.06640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.3984375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>87</v>
+      </c>
+      <c r="C3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C4" r:id="rId1" display="https://test7-internal.my.salesforce.com/00E0b000001Fm3Y" xr:uid="{EE4667ED-98A0-4458-923B-A02D1EA779B8}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2726E678-6DA9-442C-8C85-ED2905D937CF}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="16.9296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.73046875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C3" r:id="rId1" xr:uid="{A9A12091-136F-4089-AB54-51879367F8E6}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FF67A45-0B54-4944-9B39-F82B26EF60B6}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -978,7 +1386,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F105F821-5E53-4FD8-9F07-CF97205700C1}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1114,7 +1522,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC101BFC-1550-4137-B012-E4749B310065}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1249,7 +1657,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1896B5C7-9641-468E-8213-95D0BE0FBE7C}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1297,7 +1705,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{874FC87A-AF8F-49C8-9F12-715C978F4406}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -1375,657 +1783,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B029D8-A57A-4DED-8831-111F395CEFC2}">
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.06640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A5EA066-8BD7-4F60-A549-8DF4B566C85E}">
-  <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.06640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>37</v>
-      </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>43</v>
-      </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68EBF6E6-8687-4CE1-8BB6-330DEC350611}">
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.06640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" t="s">
-        <v>36</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B71B207-7F71-4F84-BC32-C3056B8DABA1}">
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.06640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" t="s">
-        <v>36</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -2089,6 +1846,657 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62B029D8-A57A-4DED-8831-111F395CEFC2}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.06640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A5EA066-8BD7-4F60-A549-8DF4B566C85E}">
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.06640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68EBF6E6-8687-4CE1-8BB6-330DEC350611}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.06640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B71B207-7F71-4F84-BC32-C3056B8DABA1}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="29.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.06640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFE25EE6-66F5-4951-9D0C-F6559D035D9C}">
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -2246,7 +2654,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B83C7FC7-2A18-436E-A373-D289D769241C}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -2415,7 +2823,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{471A3BD1-3EAB-4C67-9345-90730B6A7403}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -2583,7 +2991,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A836B93B-2094-42BE-9D92-A2EB5434CB28}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -2631,7 +3039,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB402F88-9436-4279-8D3B-028474BBC575}">
   <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -2799,7 +3207,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61C91C76-2A92-4FAB-8589-A8F89F7DC3A0}">
   <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -2833,175 +3241,6 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="C9" s="3"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF72FB96-7C2F-4711-BDC9-46D87BC44E74}">
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="1" max="1" width="7.46484375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.33203125" customWidth="1"/>
-    <col min="3" max="3" width="43.06640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" t="s">
-        <v>36</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3068,6 +3307,175 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF72FB96-7C2F-4711-BDC9-46D87BC44E74}">
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="7.46484375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.33203125" customWidth="1"/>
+    <col min="3" max="3" width="43.06640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>3</v>
+      </c>
+      <c r="B13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 

</xml_diff>